<commit_message>
Remove outdated editorial and pending-review wording
</commit_message>
<xml_diff>
--- a/reference/final_audit_documented.xlsx
+++ b/reference/final_audit_documented.xlsx
@@ -655,7 +655,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Draft rationales for Specialist 2 to review, edit, and approve; not a completed independent expert assessment.</t>
+          <t>Historical coding worksheet; final consensus labels are in Final.</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Provisional classifications and rationales for Specialist 1 to review, edit, and approve; not an independently completed expert assessment.</t>
+          <t>Historical coding worksheet; final consensus labels are in Final.</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="I2" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the user has no profile history. The stated risk is that the required recommendation input may be absent, leaving the initial user experience and expected fallback behavior undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the user has no profile history. The stated risk is that the required recommendation input may be absent, leaving the initial user experience and expected fallback behavior undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="I3" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine whether users are “similar”. The stated risk is that no similarity rule is specified, so developers cannot determine which users qualify or validate their selection. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine whether users are “similar”. The stated risk is that no similarity rule is specified, so developers cannot determine which users qualify or validate their selection. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -1859,7 +1859,7 @@
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what permission rules govern using other users’ listening paths for music discovery. The stated risk is that the story requires using other users’ listening activity without defining authorized use, leaving data eligibility and privacy boundaries unresolved. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what permission rules govern using other users’ listening paths for music discovery. The stated risk is that the story requires using other users’ listening activity without defining authorized use, leaving data eligibility and privacy boundaries unresolved. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="I5" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks through what channel and at what trigger or frequency should users receive recommendations. The stated risk is that delivery behavior is unspecified, leaving the user journey, scheduling requirements, and acceptance criteria undetermined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks through what channel and at what trigger or frequency should users receive recommendations. The stated risk is that delivery behavior is unspecified, leaving the user journey, scheduling requirements, and acceptance criteria undetermined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks how is “my area” defined and determined for a user. The stated risk is that the geographic boundary and its source are unspecified, so implementations could select different news events for the same user. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks how is “my area” defined and determined for a user. The stated risk is that the geographic boundary and its source are unspecified, so implementations could select different news events for the same user. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="I7" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what makes an international news event relevant to the user’s strictly local area. The stated risk is that the relationship between international events and local relevance is undefined, preventing consistent eligibility rules and acceptance tests. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what makes an international news event relevant to the user’s strictly local area. The stated risk is that the relationship between international events and local relevance is undefined, preventing consistent eligibility rules and acceptance tests. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2047,7 +2047,7 @@
       </c>
       <c r="I8" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criterion determines which eligible news events are “most relevant”. The stated risk is that no ranking criterion is specified, so recommendation ordering and quality cannot be objectively validated. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criterion determines which eligible news events are “most relevant”. The stated risk is that no ranking criterion is specified, so recommendation ordering and quality cannot be objectively validated. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="I9" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine which news events are “most relevant”. The stated risk is that no relevance or ranking criteria are provided, so event selection and acceptance tests lack a defined basis. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine which news events are “most relevant”. The stated risk is that no relevance or ranking criteria are provided, so event selection and acceptance tests lack a defined basis. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="I10" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what geographical relationship determines which videos appear on the map for the user’s location. The stated risk is that the story does not define how videos relate to locations or the geographical scope of matching, leaving content selection and acceptance tests undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what geographical relationship determines which videos appear on the map for the user’s location. The stated risk is that the story does not define how videos relate to locations or the geographical scope of matching, leaving content selection and acceptance tests undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="I11" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should the system determine the user’s location when it is unavailable or access to it is denied. The stated risk is that the location dependency lacks a defined fallback, leaving the map’s behavior uncertain when location cannot be obtained. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should the system determine the user’s location when it is unavailable or access to it is denied. The stated risk is that the location dependency lacks a defined fallback, leaving the map’s behavior uncertain when location cannot be obtained. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2235,7 +2235,7 @@
       </c>
       <c r="I12" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what map interaction should give the user access to a video, and what constitutes successful access. The stated risk is that “Interactive” and “access” do not define the required interaction or its testable outcome. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what map interaction should give the user access to a video, and what constitutes successful access. The stated risk is that “Interactive” and “access” do not define the required interaction or its testable outcome. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the user's location cannot be obtained. The stated risk is that no failure behavior is defined, leaving content access and the map's state unspecified when location is unavailable. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the user's location cannot be obtained. The stated risk is that no failure behavior is defined, leaving content access and the map's state unspecified when location is unavailable. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how should an admin specify the matching condition for each metric. The stated risk is that undefined comparison rules prevent determining which videos qualify and writing verifiable acceptance tests. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how should an admin specify the matching condition for each metric. The stated risk is that undefined comparison rules prevent determining which videos qualify and writing verifiable acceptance tests. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which audio and visual quality metrics must admins be able to filter by. The stated risk is that the story names no metrics, leaving the required video attributes and filter criteria undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which audio and visual quality metrics must admins be able to filter by. The stated risk is that the story names no metrics, leaving the required video attributes and filter criteria undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="I16" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should filtering treat videos whose selected quality metrics are missing or invalid. The stated risk is that undefined handling of unavailable or unusable metric values could incorrectly include or exclude videos. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should filtering treat videos whose selected quality metrics are missing or invalid. The stated risk is that undefined handling of unavailable or unusable metric values could incorrectly include or exclude videos. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="I17" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks must the assessment run before upload, or assess prior editing after the audio has been uploaded. The stated risk is that the wording leaves the processing sequence ambiguous, affecting when audio is available and where assessment belongs in the upload flow. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks must the assessment run before upload, or assess prior editing after the audio has been uploaded. The stated risk is that the wording leaves the processing sequence ambiguous, affecting when audio is available and where assessment belongs in the upload flow. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="I18" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which previously approved project policy must the assessment apply, and what rules does it contain. The stated risk is that the policy is absent, so compliance criteria and acceptance tests cannot be defined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which previously approved project policy must the assessment apply, and what rules does it contain. The stated risk is that the policy is absent, so compliance criteria and acceptance tests cannot be defined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2564,7 @@
       </c>
       <c r="I19" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what result must the admin receive when editing history or policy compliance cannot be determined. The stated risk is that undefined handling of inconclusive assessments could present uncertainty as a definitive finding. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what result must the admin receive when editing history or policy compliance cannot be determined. The stated risk is that undefined handling of inconclusive assessments could present uncertainty as a definitive finding. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="I20" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which engagement metrics should be calculated, and how is each defined. The stated risk is that neither the metrics nor their calculation rules are specified, preventing consistent implementation and verification. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which engagement metrics should be calculated, and how is each defined. The stated risk is that neither the metrics nor their calculation rules are specified, preventing consistent implementation and verification. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2658,7 @@
       </c>
       <c r="I21" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what constitutes a citizen annotation for measuring engagement. The stated risk is that the annotation unit and qualifying annotation types are undefined, so implementations could count different activities. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what constitutes a citizen annotation for measuring engagement. The stated risk is that the annotation unit and qualifying annotation types are undefined, so implementations could count different activities. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2705,7 @@
       </c>
       <c r="I22" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how should a volunteer’s experience level be determined. The stated risk is that the story does not define the evidence or criteria for experience, so implementations could assign different levels to the same volunteer. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how should a volunteer’s experience level be determined. The stated risk is that the story does not define the evidence or criteria for experience, so implementations could assign different levels to the same volunteer. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2752,7 +2752,7 @@
       </c>
       <c r="I23" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule maps a volunteer’s experience level to a reliability weight, including the permitted weight range. The stated risk is that no calculation rule or output bounds are specified, preventing reproducible calculations and verifiable acceptance tests. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule maps a volunteer’s experience level to a reliability weight, including the permitted weight range. The stated risk is that no calculation rule or output bounds are specified, preventing reproducible calculations and verifiable acceptance tests. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="I24" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule should map a volunteer’s experience level to a classification reliability weight. The stated risk is that no calculation rule is specified, so implementations could assign different weights to the same classification. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule should map a volunteer’s experience level to a classification reliability weight. The stated risk is that no calculation rule is specified, so implementations could assign different weights to the same classification. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="I25" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the experience information required for the calculation is unavailable. The stated risk is that missing input behavior is unspecified, leaving developers unable to determine whether a reliability weight can be produced. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the experience information required for the calculation is unavailable. The stated risk is that missing input behavior is unspecified, leaving developers unable to determine whether a reliability weight can be produced. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="I26" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine whether text, an image, or a video is the appropriate way to interrupt. The stated risk is that no decision rules or success criteria are provided, so the choice cannot be implemented or validated. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine whether text, an image, or a video is the appropriate way to interrupt. The stated risk is that no decision rules or success criteria are provided, so the choice cannot be implemented or validated. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="I27" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks should the feature only report the appropriate format, or also initiate the interruption. The stated risk is that the action boundary is unclear, affecting user flow and whether communication delivery is required. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks should the feature only report the appropriate format, or also initiate the interruption. The stated risk is that the action boundary is unclear, affecting user flow and whether communication delivery is required. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="I28" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what does “interrupt a volunteer” mean in this story. The stated risk is that the intended action is undefined, so the core workflow and its acceptance criteria cannot be established. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what does “interrupt a volunteer” mean in this story. The stated risk is that the intended action is undefined, so the core workflow and its acceptance criteria cannot be established. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="I29" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information should the feature use to make that determination. The stated risk is that required inputs and their sources are unspecified, leaving data requirements and the feasibility of the decision logic unresolved. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information should the feature use to make that determination. The stated risk is that required inputs and their sources are unspecified, leaving data requirements and the feasibility of the decision logic unresolved. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="I30" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what should the admin be able to do to “know when Zoonibot should comment on a subject”. The stated risk is that the intended capability is undefined, leaving no testable user outcome or functional scope. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what should the admin be able to do to “know when Zoonibot should comment on a subject”. The stated risk is that the intended capability is undefined, leaving no testable user outcome or functional scope. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="I31" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what conditions make a subject eligible for a Zoonibot comment. The stated risk is that no commenting criteria are specified, preventing implementation and validation of when a comment is warranted. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what conditions make a subject eligible for a Zoonibot comment. The stated risk is that no commenting criteria are specified, preventing implementation and validation of when a comment is warranted. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3175,7 +3175,7 @@
       </c>
       <c r="I32" s="16" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks under what conditions should Zoonibot comment again on a subject it has already commented on. The stated risk is that repeat-comment behavior is unspecified, risking unwanted duplicate comments or suppression of necessary follow-up comments. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks under what conditions should Zoonibot comment again on a subject it has already commented on. The stated risk is that repeat-comment behavior is unspecified, risking unwanted duplicate comments or suppression of necessary follow-up comments. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3222,7 +3222,7 @@
       </c>
       <c r="I33" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which aspects of a volunteer’s previous experiences should determine project recommendations. The stated risk is that the story does not define the experience data required, leaving recommendation inputs and volunteer data requirements uncertain. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which aspects of a volunteer’s previous experiences should determine project recommendations. The stated risk is that the story does not define the experience data required, leaving recommendation inputs and volunteer data requirements uncertain. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="I34" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which projects are eligible to be recommended to a volunteer. The stated risk is that the eligible project set is undefined, creating a risk of recommending projects that the volunteer cannot participate in. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which projects are eligible to be recommended to a volunteer. The stated risk is that the eligible project set is undefined, creating a risk of recommending projects that the volunteer cannot participate in. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="I35" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what counts as a volunteer’s “previous experiences” for determining recommendations. The stated risk is that the required input data and its meaning are undefined, preventing consistent recommendation logic. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what counts as a volunteer’s “previous experiences” for determining recommendations. The stated risk is that the required input data and its meaning are undefined, preventing consistent recommendation logic. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="I36" s="16" t="inlineStr">
         <is>
-          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what content and length restrictions apply to the optional description. The stated risk is that optionality alone does not establish which supplied descriptions are valid, leaving input validation and acceptance tests ambiguous. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what content and length restrictions apply to the optional description. The stated risk is that optionality alone does not establish which supplied descriptions are valid, leaving input validation and acceptance tests ambiguous. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3410,7 +3410,7 @@
       </c>
       <c r="I37" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what constraints apply to the optional description, and how should an omitted or blank description be treated. The stated risk is that description validation and the meaning of an empty value are undefined, risking inconsistent acceptance and storage. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what constraints apply to the optional description, and how should an omitted or blank description be treated. The stated risk is that description validation and the meaning of an empty value are undefined, risking inconsistent acceptance and storage. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="I38" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what actions may an estimator perform after accessing the game. The stated risk is that “Access the game” does not define participant permissions or the observable behavior required for acceptance. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what actions may an estimator perform after accessing the game. The stated risk is that “Access the game” does not define participant permissions or the observable behavior required for acceptance. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3504,7 +3504,7 @@
       </c>
       <c r="I39" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks is the invitation URL specific to a game, an individual estimator, or both. The stated risk is that the URL’s scope determines how the system identifies the intended game and recipient and prevents unintended access. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks is the invitation URL specific to a game, an individual estimator, or both. The stated risk is that the URL’s scope determines how the system identifies the intended game and recipient and prevents unintended access. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3551,7 +3551,7 @@
       </c>
       <c r="I40" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks under what conditions does an invitation URL become invalid. The stated risk is that invitation validity is undefined, preventing consistent handling and testing of expired or otherwise unusable links. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks under what conditions does an invitation URL become invalid. The stated risk is that invitation validity is undefined, preventing consistent handling and testing of expired or otherwise unusable links. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="I41" s="16" t="inlineStr">
         <is>
-          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks how should line breaks in the text field be interpreted. The stated risk is that it is unclear whether multiple lines form one item or represent separate components, which affects parsing and storage. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks how should line breaks in the text field be interpreted. The stated risk is that it is unclear whether multiple lines form one item or represent separate components, which affects parsing and storage. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
       </c>
       <c r="I42" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen if the moderator tries to start a round while another round is active. The stated risk is that the round lifecycle does not define this conflict, risking unintended overlapping rounds or replacement of an active round. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen if the moderator tries to start a round while another round is active. The stated risk is that the round lifecycle does not define this conflict, risking unintended overlapping rounds or replacement of an active round. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3692,7 +3692,7 @@
       </c>
       <c r="I43" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what action should the moderator be able to perform. The stated risk is that the story omits the requested capability, so the moderator’s workflow and functional behavior cannot be determined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what action should the moderator be able to perform. The stated risk is that the story omits the requested capability, so the moderator’s workflow and functional behavior cannot be determined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="I44" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what should happen when a moderator selects an item for estimation or re-estimation. The stated risk is that the story does not define the effect of selection, leaving the workflow and acceptance criteria undetermined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what should happen when a moderator selects an item for estimation or re-estimation. The stated risk is that the story does not define the effect of selection, leaving the workflow and acceptance criteria undetermined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
       </c>
       <c r="I45" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks which item attributes may the moderator change. The stated risk is that editable fields are unspecified, preventing definition of update behavior and validation rules. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks which item attributes may the moderator change. The stated risk is that editable fields are unspecified, preventing definition of update behavior and validation rules. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="I46" s="16" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks what restrictions, if any, apply to editing an item once estimation has begun or finished. The stated risk is that editing eligibility across estimation stages is undefined, risking changes that invalidate ongoing or completed estimates. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks what restrictions, if any, apply to editing an item once estimation has begun or finished. The stated risk is that editing eligibility across estimation stages is undefined, risking changes that invalidate ongoing or completed estimates. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="I47" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which moderators are authorized to edit a particular item. The stated risk is that the authorization scope is unspecified, risking unauthorized changes to items outside a moderator’s responsibility. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which moderators are authorized to edit a particular item. The stated risk is that the authorization scope is unspecified, risking unauthorized changes to items outside a moderator’s responsibility. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3927,7 @@
       </c>
       <c r="I48" s="16" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks at which stages of estimation is deletion permitted. The stated risk is that no lifecycle restrictions are specified, leaving deletion behavior for items undergoing or having completed estimation undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks at which stages of estimation is deletion permitted. The stated risk is that no lifecycle restrictions are specified, leaving deletion behavior for items undergoing or having completed estimation undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="I49" s="16" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks what should happen to existing estimates associated with a deleted item. The stated risk is that the treatment of related estimates is unspecified, risking orphaned data or unintended loss of estimation history. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks what should happen to existing estimates associated with a deleted item. The stated risk is that the treatment of related estimates is unspecified, risking orphaned data or unintended loss of estimation history. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="I50" s="16" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks if an item already has estimation data, what should happen to that data when the item is deleted. The stated risk is that the treatment of potentially associated data is undefined, risking orphaned records or unintended loss of estimates. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks if an item already has estimation data, what should happen to that data when the item is deleted. The stated risk is that the treatment of potentially associated data is undefined, risking orphaned records or unintended loss of estimates. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="I51" s="16" t="inlineStr">
         <is>
-          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what makes an estimate value “adequate,” including its unit, permitted format, and valid range. The stated risk is that “Adequate” provides no testable validation rule, so implementations could accept incompatible or invalid values. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what makes an estimate value “adequate,” including its unit, permitted format, and valid range. The stated risk is that “Adequate” provides no testable validation rule, so implementations could accept incompatible or invalid values. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="I52" s="16" t="inlineStr">
         <is>
-          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what unit and allowed values must the estimate use. The stated risk is that the estimate’s representation is unspecified, preventing consistent storage and input validation. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what unit and allowed values must the estimate use. The stated risk is that the estimate’s representation is unspecified, preventing consistent storage and input validation. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4162,7 +4162,7 @@
       </c>
       <c r="I53" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what should happen to stories when a moderator imports them from a spreadsheet. The stated risk is that the intended outcome is unspecified, preventing definition of the feature’s behavior and acceptance criteria. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what should happen to stories when a moderator imports them from a spreadsheet. The stated risk is that the intended outcome is unspecified, preventing definition of the feature’s behavior and acceptance criteria. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
       </c>
       <c r="I54" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks at what stage of a game must its transcript be available for viewing. The stated risk is that availability during or after a game is undefined, leaving transcript lifecycle and update behavior uncertain. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks at what stage of a game must its transcript be available for viewing. The stated risk is that availability during or after a game is undefined, leaving transcript lifecycle and update behavior uncertain. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4256,7 +4256,7 @@
       </c>
       <c r="I55" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how does the user identify which game’s transcript to view. The stated risk is that the target-game selection flow is unspecified, preventing implementation and validation of the viewing journey. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how does the user identify which game’s transcript to view. The stated risk is that the target-game selection flow is unspecified, preventing implementation and validation of the viewing journey. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4303,7 +4303,7 @@
       </c>
       <c r="I56" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks which actions must the moderator be able to perform on user credentials. The stated risk is that “Manage” does not specify supported operations, so implementation scope and acceptance tests cannot be determined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks which actions must the moderator be able to perform on user credentials. The stated risk is that “Manage” does not specify supported operations, so implementation scope and acceptance tests cannot be determined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4350,7 +4350,7 @@
       </c>
       <c r="I57" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information must a game transcript contain. The stated risk is that undefined transcript contents prevent determining which game data must be exported and testing completeness. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information must a game transcript contain. The stated risk is that undefined transcript contents prevent determining which game data must be exported and testing completeness. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="I58" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks which terminology and conventions from the previous sprint must the sponsor list follow. The stated risk is that the referenced conventions are absent from the story, so required wording and behavior cannot be implemented or verified. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks which terminology and conventions from the previous sprint must the sponsor list follow. The stated risk is that the referenced conventions are absent from the story, so required wording and behavior cannot be implemented or verified. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="I59" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what is the authoritative source of the sponsor list. The stated risk is that the story does not identify where sponsor records originate, leaving data retrieval and correctness validation undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what is the authoritative source of the sponsor list. The stated risk is that the story does not identify where sponsor records originate, leaving data retrieval and correctness validation undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="I60" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should an anonymous user see when the sponsor list is empty or cannot be retrieved. The stated risk is that empty and failure behavior are unspecified, preventing consistent handling and verification of these distinct outcomes. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should an anonymous user see when the sponsor list is empty or cannot be retrieved. The stated risk is that empty and failure behavior are unspecified, preventing consistent handling and verification of these distinct outcomes. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="I61" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which user profiles and profile fields may an anonymous user view. The stated risk is that the list’s scope and visible data are unspecified, preventing access-control and privacy requirements from being tested. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which user profiles and profile fields may an anonymous user view. The stated risk is that the list’s scope and visible data are unspecified, preventing access-control and privacy requirements from being tested. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="I62" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what must anonymous users see when the profile list cannot be retrieved. The stated risk is that retrieval failure behavior is undefined, so users could receive a misleading empty list or an indefinite loading state. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what must anonymous users see when the profile list cannot be retrieved. The stated risk is that retrieval failure behavior is undefined, so users could receive a misleading empty list or an indefinite loading state. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4632,7 +4632,7 @@
       </c>
       <c r="I63" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what spatial information must the map show to locate buildings and rooms. The stated risk is that the story does not specify whether room locations require floor identification, interior layouts, or other spatial relationships, leaving the map’s data requirements uncertain. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what spatial information must the map show to locate buildings and rooms. The stated risk is that the story does not specify whether room locations require floor identification, interior layouts, or other spatial relationships, leaving the map’s data requirements uncertain. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="I64" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks does a waitlist entry apply to an entire training or to a particular scheduled session. The stated risk is that the waitlist’s scope is undefined, risking enrollment against the wrong training occurrence. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks does a waitlist entry apply to an entire training or to a particular scheduled session. The stated risk is that the waitlist’s scope is undefined, risking enrollment against the wrong training occurrence. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4726,7 +4726,7 @@
       </c>
       <c r="I65" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what determines the “appropriate order” of trainings, including how ties are resolved. The stated risk is that no ordering rule is defined, so developers cannot implement or test the intended sequence. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what determines the “appropriate order” of trainings, including how ties are resolved. The stated risk is that no ordering rule is defined, so developers cannot implement or test the intended sequence. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4773,7 +4773,7 @@
       </c>
       <c r="I66" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the trainee see when the prerequisite has not been completed. The stated risk is that the blocked state is unspecified, leaving developers unable to determine the required interface behavior or validate that the visibility restriction is satisfied. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the trainee see when the prerequisite has not been completed. The stated risk is that the blocked state is unspecified, leaving developers unable to determine the required interface behavior or validate that the visibility restriction is satisfied. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4820,7 +4820,7 @@
       </c>
       <c r="I67" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule determines whether two venue records are duplicates. The stated risk is that undefined identity and uniqueness rules could allow duplicate venues or reject distinct venues. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule determines whether two venue records are duplicates. The stated risk is that undefined identity and uniqueness rules could allow duplicate venues or reject distinct venues. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="I68" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information is required to create a venue. The stated risk is that missing required attributes prevent defining the data model and testing whether a venue record is complete. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information is required to create a venue. The stated risk is that missing required attributes prevent defining the data model and testing whether a venue record is complete. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4914,7 @@
       </c>
       <c r="I69" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules does the previously approved project policy impose on creating and maintaining venues. The stated risk is that the referenced policy is absent, so policy compliance cannot be implemented or verified. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules does the previously approved project policy impose on creating and maintaining venues. The stated risk is that the referenced policy is absent, so policy compliance cannot be implemented or verified. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -4961,7 +4961,7 @@
       </c>
       <c r="I70" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how does an anonymous user identify the venue whose details they want to view. The stated risk is that the entry point and venue selection flow are unspecified, leaving the viewing journey incomplete. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how does an anonymous user identify the venue whose details they want to view. The stated risk is that the entry point and venue selection flow are unspecified, leaving the viewing journey incomplete. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="I71" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks how does an anonymous user reach the details of a specific venue. The stated risk is that the entry point and venue selection flow are unspecified, preventing definition of the required navigation and venue identification behavior. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks how does an anonymous user reach the details of a specific venue. The stated risk is that the entry point and venue selection flow are unspecified, preventing definition of the required navigation and venue identification behavior. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="I72" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which venues must a training coordinator be able to view. The stated risk is that the eligible venue set is unspecified, preventing definition of retrieval scope and tests for venue inclusion or exclusion. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which venues must a training coordinator be able to view. The stated risk is that the eligible venue set is unspecified, preventing definition of retrieval scope and tests for venue inclusion or exclusion. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="I73" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks does creating a blog post save it as a draft or immediately make it publicly visible. The stated risk is that the initial post state and visibility are undefined, risking unintended publication and conflicting acceptance tests. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks does creating a blog post save it as a draft or immediately make it publicly visible. The stated risk is that the initial post state and visibility are undefined, risking unintended publication and conflicting acceptance tests. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5149,7 +5149,7 @@
       </c>
       <c r="I74" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the administrator experience when a blog post cannot be saved. The stated risk is that failure behavior and preservation of entered content are unspecified, risking silent failures, lost work, or duplicate posts during retries. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the administrator experience when a blog post cannot be saved. The stated risk is that failure behavior and preservation of entered content are unspecified, risking silent failures, lost work, or duplicate posts during retries. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="I75" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what content is required for a valid blog post. The stated risk is that required fields and content constraints are unspecified, preventing definition of the data model and validation criteria. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what content is required for a valid blog post. The stated risk is that required fields and content constraints are unspecified, preventing definition of the data model and validation criteria. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="I76" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks who qualifies as a sponsor, and what determines their permission to create blog posts. The stated risk is that the actor and authorization rules are undefined, so eligibility checks and access-control tests cannot be established. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks who qualifies as a sponsor, and what determines their permission to create blog posts. The stated risk is that the actor and authorization rules are undefined, so eligibility checks and access-control tests cannot be established. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5290,7 +5290,7 @@
       </c>
       <c r="I77" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information must a blog post contain to be created successfully. The stated risk is that required content and attributes are unspecified, preventing a defined data model and testable creation criteria. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information must a blog post contain to be created successfully. The stated risk is that required content and attributes are unspecified, preventing a defined data model and testable creation criteria. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5337,7 +5337,7 @@
       </c>
       <c r="I78" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules, if any, limit registration by deadline or summit capacity. The stated risk is that acceptance limits are undefined, so registration could be accepted when business rules require rejection. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules, if any, limit registration by deadline or summit capacity. The stated risk is that acceptance limits are undefined, so registration could be accepted when business rules require rejection. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5384,7 +5384,7 @@
       </c>
       <c r="I79" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what actions must an attendee complete for registration to be considered successful. The stated risk is that the registration scope and completion state are undefined, leaving developers unable to distinguish an initiated registration from a completed one. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what actions must an attendee complete for registration to be considered successful. The stated risk is that the registration scope and completion state are undefined, leaving developers unable to distinguish an initiated registration from a completed one. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5431,7 @@
       </c>
       <c r="I80" s="16" t="inlineStr">
         <is>
-          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what outcome marks registration as successfully completed. The stated risk is that the story provides no observable completion criterion, so implementation and tests cannot distinguish a submitted request from a completed registration. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what outcome marks registration as successfully completed. The stated risk is that the story provides no observable completion criterion, so implementation and tests cannot distinguish a submitted request from a completed registration. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5478,7 +5478,7 @@
       </c>
       <c r="I81" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what schedule does “the schedule” refer to. The stated risk is that the schedule’s subject and source are undefined, so developers cannot determine which data to retrieve. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what schedule does “the schedule” refer to. The stated risk is that the schedule’s subject and source are undefined, so developers cannot determine which data to retrieve. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5525,7 +5525,7 @@
       </c>
       <c r="I82" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what user action is intended by “something about see the schedule”. The stated risk is that the wording does not establish the required behavior, preventing a testable definition of successful use. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what user action is intended by “something about see the schedule”. The stated risk is that the wording does not establish the required behavior, preventing a testable definition of successful use. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5572,7 +5572,7 @@
       </c>
       <c r="I83" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what video input must be supported: prerecorded video, a live stream, or both. The stated risk is that the input lifecycle determines whether processing operates on a complete timeline or must handle incoming frames continuously. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what video input must be supported: prerecorded video, a live stream, or both. The stated risk is that the input lifecycle determines whether processing operates on a complete timeline or must handle incoming frames continuously. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5619,7 +5619,7 @@
       </c>
       <c r="I84" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what should each music recommendation contain. The stated risk is that the recommended entity and required output information are unspecified, leaving the result data model and acceptance criteria undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what should each music recommendation contain. The stated risk is that the recommended entity and required output information are unspecified, leaving the result data model and acceptance criteria undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="I85" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which music catalog should supply the recommendations. The stated risk is that the source and boundaries of eligible music are unspecified, leaving data availability and external dependencies unresolved. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which music catalog should supply the recommendations. The stated risk is that the source and boundaries of eligible music are unspecified, leaving data availability and external dependencies unresolved. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5713,7 +5713,7 @@
       </c>
       <c r="I86" s="16" t="inlineStr">
         <is>
-          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what observable condition establishes that the prerequisite story has been completed. The stated risk is that “Completed” lacks a testable definition, leaving the upload eligibility rule undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what observable condition establishes that the prerequisite story has been completed. The stated risk is that “Completed” lacks a testable definition, leaving the upload eligibility rule undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="I87" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when a user attempts to upload an image before the prerequisite is completed. The stated risk is that the blocked interaction and failure response are unspecified, preventing consistent enforcement and acceptance testing. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when a user attempts to upload an image before the prerequisite is completed. The stated risk is that the blocked interaction and failure response are unspecified, preventing consistent enforcement and acceptance testing. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5807,7 +5807,7 @@
       </c>
       <c r="I88" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which users’ credentials may an admin manage. The stated risk is that the authorization scope is unspecified, risking unauthorized changes to credentials. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which users’ credentials may an admin manage. The stated risk is that the authorization scope is unspecified, risking unauthorized changes to credentials. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5854,7 +5854,7 @@
       </c>
       <c r="I89" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what defines a segmentation boundary in a video. The stated risk is that without a definition, developers cannot determine which detected points qualify as boundaries or validate segmentation correctness. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what defines a segmentation boundary in a video. The stated risk is that without a definition, developers cannot determine which detected points qualify as boundaries or validate segmentation correctness. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5901,7 +5901,7 @@
       </c>
       <c r="I90" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks must this feature generate automated segmentation boundaries, or display boundaries already produced elsewhere. The stated risk is that the story does not establish whether automated segmentation processing is part of the feature, leaving its scope and dependencies undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks must this feature generate automated segmentation boundaries, or display boundaries already produced elsewhere. The stated risk is that the story does not establish whether automated segmentation processing is part of the feature, leaving its scope and dependencies undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="I91" s="16" t="inlineStr">
         <is>
-          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what maximum elapsed time is acceptable from the admin requesting the boundaries to their being visible. The stated risk is that “As fast as necessary” supplies no measurable performance target, making response-time acceptance tests impossible to define. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what maximum elapsed time is acceptable from the admin requesting the boundaries to their being visible. The stated risk is that “As fast as necessary” supplies no measurable performance target, making response-time acceptance tests impossible to define. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="I92" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the admin see when automated segmentation boundaries are unavailable. The stated risk is that the missing unavailable-result behavior could cause an unprocessed video or failed segmentation to appear indistinguishable from a valid result with no boundaries. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the admin see when automated segmentation boundaries are unavailable. The stated risk is that the missing unavailable-result behavior could cause an unprocessed video or failed segmentation to appear indistinguishable from a valid result with no boundaries. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6042,7 +6042,7 @@
       </c>
       <c r="I93" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what constitutes a segmentation boundary in this story. The stated risk is that the boundary’s meaning is undefined, leaving its data representation and acceptance criteria uncertain. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what constitutes a segmentation boundary in this story. The stated risk is that the boundary’s meaning is undefined, leaving its data representation and acceptance criteria uncertain. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="I94" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what must happen when a clip fails validation. The stated risk is that the failure outcome and subsequent workflow are unspecified, leaving unsuccessful validation without defined behavior. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what must happen when a clip fails validation. The stated risk is that the failure outcome and subsequent workflow are unspecified, leaving unsuccessful validation without defined behavior. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6136,7 @@
       </c>
       <c r="I95" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules must edited timestamps satisfy regarding video duration, segment order, overlaps, and gaps. The stated risk is that missing validation rules could allow invalid boundaries or reject legitimate corrections. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules must edited timestamps satisfy regarding video duration, segment order, overlaps, and gaps. The stated risk is that missing validation rules could allow invalid boundaries or reject legitimate corrections. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6183,7 +6183,7 @@
       </c>
       <c r="I96" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which timestamps should the user be able to edit for each segment. The stated risk is that the editable timestamp fields are unspecified, preventing definition of the editing controls and update behavior. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which timestamps should the user be able to edit for each segment. The stated risk is that the editable timestamp fields are unspecified, preventing definition of the editing controls and update behavior. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6230,7 +6230,7 @@
       </c>
       <c r="I97" s="16" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks when further contrasting annotations arrive for an already alerted subject, should another alert be generated. The stated risk is that undefined repeat-trigger behavior could produce duplicate alerts or suppress subsequent conflicts. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks when further contrasting annotations arrive for an already alerted subject, should another alert be generated. The stated risk is that undefined repeat-trigger behavior could produce duplicate alerts or suppress subsequent conflicts. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6277,7 +6277,7 @@
       </c>
       <c r="I98" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what should happen to an image when it is automatically “isolated”. The stated risk is that “Isolate” does not define the required action or the image’s resulting availability, leaving the core behavior untestable. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what should happen to an image when it is automatically “isolated”. The stated risk is that “Isolate” does not define the required action or the image’s resulting availability, leaving the core behavior untestable. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6324,7 +6324,7 @@
       </c>
       <c r="I99" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should the system handle images whose animal presence cannot be determined confidently. The stated risk is that undefined handling of uncertain images could isolate images containing animals or leave qualifying images unprocessed. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should the system handle images whose animal presence cannot be determined confidently. The stated risk is that undefined handling of uncertain images could isolate images containing animals or leave qualifying images unprocessed. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6371,7 +6371,7 @@
       </c>
       <c r="I100" s="16" t="inlineStr">
         <is>
-          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what results must the counter return, and in what format. The stated risk is that the story does not define the output contract, preventing validation that the results meet the user's intended use. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what results must the counter return, and in what format. The stated risk is that the story does not define the output contract, preventing validation that the results meet the user's intended use. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="I101" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which Snapshot Serengeti images must be processed. The stated risk is that the image population is unspecified, leaving processing scope and workload undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which Snapshot Serengeti images must be processed. The stated risk is that the image population is unspecified, leaving processing scope and workload undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -13145,7 +13145,7 @@
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks through what channel and at what trigger or frequency should users receive recommendations. The stated risk is that delivery behavior is unspecified, leaving the user journey, scheduling requirements, and acceptance criteria undetermined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks through what channel and at what trigger or frequency should users receive recommendations. The stated risk is that delivery behavior is unspecified, leaving the user journey, scheduling requirements, and acceptance criteria undetermined. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K2" s="8" t="inlineStr">
@@ -13165,7 +13165,7 @@
       </c>
       <c r="N2" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The clarification focuses on delivery conditions and observable timing; without them, a basic acceptance test for receiving recommendations cannot be defined.</t>
+          <t>The clarification focuses on delivery conditions and observable timing; without them, a basic acceptance test for receiving recommendations cannot be defined.</t>
         </is>
       </c>
     </row>
@@ -13217,7 +13217,7 @@
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks how is “my area” defined and determined for a user. The stated risk is that the geographic boundary and its source are unspecified, so implementations could select different news events for the same user. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks how is “my area” defined and determined for a user. The stated risk is that the geographic boundary and its source are unspecified, so implementations could select different news events for the same user. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K3" s="8" t="inlineStr">
@@ -13237,7 +13237,7 @@
       </c>
       <c r="N3" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): “My area” admits several geographic interpretations (city, radius, administrative boundary); the ambiguity itself is the central defect.</t>
+          <t>“My area” admits several geographic interpretations (city, radius, administrative boundary); the ambiguity itself is the central defect.</t>
         </is>
       </c>
     </row>
@@ -13289,7 +13289,7 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what makes an international news event relevant to the user’s strictly local area. The stated risk is that the relationship between international events and local relevance is undefined, preventing consistent eligibility rules and acceptance tests. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what makes an international news event relevant to the user’s strictly local area. The stated risk is that the relationship between international events and local relevance is undefined, preventing consistent eligibility rules and acceptance tests. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K4" s="8" t="inlineStr">
@@ -13309,7 +13309,7 @@
       </c>
       <c r="N4" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): “Relevant to the strictly local area” can mean geographic proximity, local impact, or audience relevance, producing conflicting interpretations.</t>
+          <t>“Relevant to the strictly local area” can mean geographic proximity, local impact, or audience relevance, producing conflicting interpretations.</t>
         </is>
       </c>
     </row>
@@ -13361,7 +13361,7 @@
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine which news events are “most relevant”. The stated risk is that no relevance or ranking criteria are provided, so event selection and acceptance tests lack a defined basis. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine which news events are “most relevant”. The stated risk is that no relevance or ranking criteria are provided, so event selection and acceptance tests lack a defined basis. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K5" s="8" t="inlineStr">
@@ -13381,7 +13381,7 @@
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Ranking by “most relevant” requires an undefined domain-specific relevance rule; testability is a consequence of this missing rule.</t>
+          <t>Ranking by “most relevant” requires an undefined domain-specific relevance rule; testability is a consequence of this missing rule.</t>
         </is>
       </c>
     </row>
@@ -13433,7 +13433,7 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what map interaction should give the user access to a video, and what constitutes successful access. The stated risk is that “Interactive” and “access” do not define the required interaction or its testable outcome. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what map interaction should give the user access to a video, and what constitutes successful access. The stated risk is that “Interactive” and “access” do not define the required interaction or its testable outcome. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
@@ -13453,7 +13453,7 @@
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The question seeks an observable map interaction and success condition needed to test whether video access works.</t>
+          <t>The question seeks an observable map interaction and success condition needed to test whether video access works.</t>
         </is>
       </c>
     </row>
@@ -13505,7 +13505,7 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how should an admin specify the matching condition for each metric. The stated risk is that undefined comparison rules prevent determining which videos qualify and writing verifiable acceptance tests. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how should an admin specify the matching condition for each metric. The stated risk is that undefined comparison rules prevent determining which videos qualify and writing verifiable acceptance tests. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K7" s="8" t="inlineStr">
@@ -13525,7 +13525,7 @@
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The matching semantics for each quality metric are missing domain rules; this is not merely a lack of a test case.</t>
+          <t>The matching semantics for each quality metric are missing domain rules; this is not merely a lack of a test case.</t>
         </is>
       </c>
     </row>
@@ -13577,7 +13577,7 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule maps a volunteer’s experience level to a reliability weight, including the permitted weight range. The stated risk is that no calculation rule or output bounds are specified, preventing reproducible calculations and verifiable acceptance tests. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule maps a volunteer’s experience level to a reliability weight, including the permitted weight range. The stated risk is that no calculation rule or output bounds are specified, preventing reproducible calculations and verifiable acceptance tests. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr">
@@ -13597,7 +13597,7 @@
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The mapping from experience to reliability weight is central to the requested classification logic; the numeric range is a secondary detail.</t>
+          <t>The mapping from experience to reliability weight is central to the requested classification logic; the numeric range is a secondary detail.</t>
         </is>
       </c>
     </row>
@@ -13649,7 +13649,7 @@
       </c>
       <c r="J9" s="8" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule should map a volunteer’s experience level to a classification reliability weight. The stated risk is that no calculation rule is specified, so implementations could assign different weights to the same classification. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule should map a volunteer’s experience level to a classification reliability weight. The stated risk is that no calculation rule is specified, so implementations could assign different weights to the same classification. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K9" s="8" t="inlineStr">
@@ -13669,7 +13669,7 @@
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The core transformation from experience level to reliability weight is unspecified, making the required domain behavior indeterminate.</t>
+          <t>The core transformation from experience level to reliability weight is unspecified, making the required domain behavior indeterminate.</t>
         </is>
       </c>
     </row>
@@ -13721,7 +13721,7 @@
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what does “interrupt a volunteer” mean in this story. The stated risk is that the intended action is undefined, so the core workflow and its acceptance criteria cannot be established. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what does “interrupt a volunteer” mean in this story. The stated risk is that the intended action is undefined, so the core workflow and its acceptance criteria cannot be established. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
@@ -13741,7 +13741,7 @@
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): “Interrupt” is a polysemous verb and could refer to notifying, pausing, or blocking a volunteer; the central problem is ambiguity.</t>
+          <t>“Interrupt” is a polysemous verb and could refer to notifying, pausing, or blocking a volunteer; the central problem is ambiguity.</t>
         </is>
       </c>
     </row>
@@ -13793,7 +13793,7 @@
       </c>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what should the admin be able to do to “know when Zoonibot should comment on a subject”. The stated risk is that the intended capability is undefined, leaving no testable user outcome or functional scope. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what should the admin be able to do to “know when Zoonibot should comment on a subject”. The stated risk is that the intended capability is undefined, leaving no testable user outcome or functional scope. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K11" s="8" t="inlineStr">
@@ -13813,7 +13813,7 @@
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The story does not specify the admin-facing action or outcome implied by “know when”; this is missing core functionality.</t>
+          <t>The story does not specify the admin-facing action or outcome implied by “know when”; this is missing core functionality.</t>
         </is>
       </c>
     </row>
@@ -13865,7 +13865,7 @@
       </c>
       <c r="J12" s="8" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks under what conditions should Zoonibot comment again on a subject it has already commented on. The stated risk is that repeat-comment behavior is unspecified, risking unwanted duplicate comments or suppression of necessary follow-up comments. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks under what conditions should Zoonibot comment again on a subject it has already commented on. The stated risk is that repeat-comment behavior is unspecified, risking unwanted duplicate comments or suppression of necessary follow-up comments. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -13885,7 +13885,7 @@
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The repeat-comment policy is part of the bot’s core decision logic, rather than a peripheral downstream consistency constraint.</t>
+          <t>The repeat-comment policy is part of the bot’s core decision logic, rather than a peripheral downstream consistency constraint.</t>
         </is>
       </c>
     </row>
@@ -13937,7 +13937,7 @@
       </c>
       <c r="J13" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what counts as a volunteer’s “previous experiences” for determining recommendations. The stated risk is that the required input data and its meaning are undefined, preventing consistent recommendation logic. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what counts as a volunteer’s “previous experiences” for determining recommendations. The stated risk is that the required input data and its meaning are undefined, preventing consistent recommendation logic. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K13" s="8" t="inlineStr">
@@ -13957,7 +13957,7 @@
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): “Previous experiences” can denote completed tasks, projects, ratings, or interactions; multiple plausible interpretations remain.</t>
+          <t>“Previous experiences” can denote completed tasks, projects, ratings, or interactions; multiple plausible interpretations remain.</t>
         </is>
       </c>
     </row>
@@ -14009,7 +14009,7 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what content and length restrictions apply to the optional description. The stated risk is that optionality alone does not establish which supplied descriptions are valid, leaving input validation and acceptance tests ambiguous. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what content and length restrictions apply to the optional description. The stated risk is that optionality alone does not establish which supplied descriptions are valid, leaving input validation and acceptance tests ambiguous. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr">
@@ -14029,7 +14029,7 @@
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The question primarily requests field length and content constraints for an optional description, rather than the core acceptance outcome.</t>
+          <t>The question primarily requests field length and content constraints for an optional description, rather than the core acceptance outcome.</t>
         </is>
       </c>
     </row>
@@ -14081,7 +14081,7 @@
       </c>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what actions may an estimator perform after accessing the game. The stated risk is that “Access the game” does not define participant permissions or the observable behavior required for acceptance. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what actions may an estimator perform after accessing the game. The stated risk is that “Access the game” does not define participant permissions or the observable behavior required for acceptance. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K15" s="8" t="inlineStr">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The permitted estimator actions constitute the core functional scope after game access; no action set is defined.</t>
+          <t>The permitted estimator actions constitute the core functional scope after game access; no action set is defined.</t>
         </is>
       </c>
     </row>
@@ -14153,7 +14153,7 @@
       </c>
       <c r="J16" s="8" t="inlineStr">
         <is>
-          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks how should line breaks in the text field be interpreted. The stated risk is that it is unclear whether multiple lines form one item or represent separate components, which affects parsing and storage. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks how should line breaks in the text field be interpreted. The stated risk is that it is unclear whether multiple lines form one item or represent separate components, which affects parsing and storage. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K16" s="8" t="inlineStr">
@@ -14173,7 +14173,7 @@
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The question targets exact text-field parsing semantics for line breaks, a low-level format and validation issue.</t>
+          <t>The question targets exact text-field parsing semantics for line breaks, a low-level format and validation issue.</t>
         </is>
       </c>
     </row>
@@ -14225,7 +14225,7 @@
       </c>
       <c r="J17" s="8" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen if the moderator tries to start a round while another round is active. The stated risk is that the round lifecycle does not define this conflict, risking unintended overlapping rounds or replacement of an active round. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen if the moderator tries to start a round while another round is active. The stated risk is that the round lifecycle does not define this conflict, risking unintended overlapping rounds or replacement of an active round. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K17" s="8" t="inlineStr">
@@ -14245,7 +14245,7 @@
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The question asks for the invalid-state response when a second round is started, rather than record consistency across entities.</t>
+          <t>The question asks for the invalid-state response when a second round is started, rather than record consistency across entities.</t>
         </is>
       </c>
     </row>
@@ -14297,7 +14297,7 @@
       </c>
       <c r="J18" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what should happen when a moderator selects an item for estimation or re-estimation. The stated risk is that the story does not define the effect of selection, leaving the workflow and acceptance criteria undetermined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what should happen when a moderator selects an item for estimation or re-estimation. The stated risk is that the story does not define the effect of selection, leaving the workflow and acceptance criteria undetermined. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr">
@@ -14317,7 +14317,7 @@
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Selecting an item for estimation lacks a defined resulting user-visible action, a core behavior gap.</t>
+          <t>Selecting an item for estimation lacks a defined resulting user-visible action, a core behavior gap.</t>
         </is>
       </c>
     </row>
@@ -14369,7 +14369,7 @@
       </c>
       <c r="J19" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks which item attributes may the moderator change. The stated risk is that editable fields are unspecified, preventing definition of update behavior and validation rules. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks which item attributes may the moderator change. The stated risk is that editable fields are unspecified, preventing definition of update behavior and validation rules. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K19" s="8" t="inlineStr">
@@ -14389,7 +14389,7 @@
       </c>
       <c r="N19" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The attributes the moderator may edit define the core edit operation; the missing action scope is more direct than broader domain context.</t>
+          <t>The attributes the moderator may edit define the core edit operation; the missing action scope is more direct than broader domain context.</t>
         </is>
       </c>
     </row>
@@ -14441,7 +14441,7 @@
       </c>
       <c r="J20" s="8" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks what restrictions, if any, apply to editing an item once estimation has begun or finished. The stated risk is that editing eligibility across estimation stages is undefined, risking changes that invalidate ongoing or completed estimates. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks what restrictions, if any, apply to editing an item once estimation has begun or finished. The stated risk is that editing eligibility across estimation stages is undefined, risking changes that invalidate ongoing or completed estimates. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K20" s="8" t="inlineStr">
@@ -14461,7 +14461,7 @@
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Allowed editing stages define the validity of the principal edit action; this is a core lifecycle business rule.</t>
+          <t>Allowed editing stages define the validity of the principal edit action; this is a core lifecycle business rule.</t>
         </is>
       </c>
     </row>
@@ -14513,7 +14513,7 @@
       </c>
       <c r="J21" s="8" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks at which stages of estimation is deletion permitted. The stated risk is that no lifecycle restrictions are specified, leaving deletion behavior for items undergoing or having completed estimation undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks at which stages of estimation is deletion permitted. The stated risk is that no lifecycle restrictions are specified, leaving deletion behavior for items undergoing or having completed estimation undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K21" s="8" t="inlineStr">
@@ -14533,7 +14533,7 @@
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Deletion eligibility at each estimation stage is an essential business rule governing the requested deletion behavior.</t>
+          <t>Deletion eligibility at each estimation stage is an essential business rule governing the requested deletion behavior.</t>
         </is>
       </c>
     </row>
@@ -14585,7 +14585,7 @@
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks what should happen to existing estimates associated with a deleted item. The stated risk is that the treatment of related estimates is unspecified, risking orphaned data or unintended loss of estimation history. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks what should happen to existing estimates associated with a deleted item. The stated risk is that the treatment of related estimates is unspecified, risking orphaned data or unintended loss of estimation history. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K22" s="8" t="inlineStr">
@@ -14605,7 +14605,7 @@
       </c>
       <c r="N22" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Handling estimates linked to a deleted item is a downstream referential and transactional integrity concern.</t>
+          <t>Handling estimates linked to a deleted item is a downstream referential and transactional integrity concern.</t>
         </is>
       </c>
     </row>
@@ -14657,7 +14657,7 @@
       </c>
       <c r="J23" s="8" t="inlineStr">
         <is>
-          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what makes an estimate value “adequate,” including its unit, permitted format, and valid range. The stated risk is that “Adequate” provides no testable validation rule, so implementations could accept incompatible or invalid values. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what makes an estimate value “adequate,” including its unit, permitted format, and valid range. The stated risk is that “Adequate” provides no testable validation rule, so implementations could accept incompatible or invalid values. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K23" s="8" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): “Adequate” requires a domain-specific definition of an acceptable estimate; units and format are supporting details.</t>
+          <t>“Adequate” requires a domain-specific definition of an acceptable estimate; units and format are supporting details.</t>
         </is>
       </c>
     </row>
@@ -14729,7 +14729,7 @@
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what should happen to stories when a moderator imports them from a spreadsheet. The stated risk is that the intended outcome is unspecified, preventing definition of the feature’s behavior and acceptance criteria. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what should happen to stories when a moderator imports them from a spreadsheet. The stated risk is that the intended outcome is unspecified, preventing definition of the feature’s behavior and acceptance criteria. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K24" s="8" t="inlineStr">
@@ -14749,7 +14749,7 @@
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The import operation lacks its principal observable effect on stories, a missing core action outcome.</t>
+          <t>The import operation lacks its principal observable effect on stories, a missing core action outcome.</t>
         </is>
       </c>
     </row>
@@ -14801,7 +14801,7 @@
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks which actions must the moderator be able to perform on user credentials. The stated risk is that “Manage” does not specify supported operations, so implementation scope and acceptance tests cannot be determined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks which actions must the moderator be able to perform on user credentials. The stated risk is that “Manage” does not specify supported operations, so implementation scope and acceptance tests cannot be determined. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K25" s="8" t="inlineStr">
@@ -14821,7 +14821,7 @@
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The set of credential-management operations defines the primary user-visible functionality.</t>
+          <t>The set of credential-management operations defines the primary user-visible functionality.</t>
         </is>
       </c>
     </row>
@@ -14873,7 +14873,7 @@
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks which terminology and conventions from the previous sprint must the sponsor list follow. The stated risk is that the referenced conventions are absent from the story, so required wording and behavior cannot be implemented or verified. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks which terminology and conventions from the previous sprint must the sponsor list follow. The stated risk is that the referenced conventions are absent from the story, so required wording and behavior cannot be implemented or verified. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K26" s="8" t="inlineStr">
@@ -14893,7 +14893,7 @@
       </c>
       <c r="N26" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The referenced prior-sprint conventions are missing external domain context rather than an ambiguous term with two explicit readings.</t>
+          <t>The referenced prior-sprint conventions are missing external domain context rather than an ambiguous term with two explicit readings.</t>
         </is>
       </c>
     </row>
@@ -14945,7 +14945,7 @@
       </c>
       <c r="J27" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks how does an anonymous user reach the details of a specific venue. The stated risk is that the entry point and venue selection flow are unspecified, preventing definition of the required navigation and venue identification behavior. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks how does an anonymous user reach the details of a specific venue. The stated risk is that the entry point and venue selection flow are unspecified, preventing definition of the required navigation and venue identification behavior. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K27" s="8" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The navigation path to a venue’s details is an unspecified core user interaction, not just a missing test assertion.</t>
+          <t>The navigation path to a venue’s details is an unspecified core user interaction, not just a missing test assertion.</t>
         </is>
       </c>
     </row>
@@ -15017,7 +15017,7 @@
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks does creating a blog post save it as a draft or immediately make it publicly visible. The stated risk is that the initial post state and visibility are undefined, risking unintended publication and conflicting acceptance tests. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks does creating a blog post save it as a draft or immediately make it publicly visible. The stated risk is that the initial post state and visibility are undefined, risking unintended publication and conflicting acceptance tests. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K28" s="8" t="inlineStr">
@@ -15037,7 +15037,7 @@
       </c>
       <c r="N28" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Draft versus immediate publication are two conflicting interpretations of the result of creating a post.</t>
+          <t>Draft versus immediate publication are two conflicting interpretations of the result of creating a post.</t>
         </is>
       </c>
     </row>
@@ -15089,7 +15089,7 @@
       </c>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules, if any, limit registration by deadline or summit capacity. The stated risk is that acceptance limits are undefined, so registration could be accepted when business rules require rejection. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules, if any, limit registration by deadline or summit capacity. The stated risk is that acceptance limits are undefined, so registration could be accepted when business rules require rejection. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K29" s="8" t="inlineStr">
@@ -15109,7 +15109,7 @@
       </c>
       <c r="N29" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Registration deadlines and capacity limits are core eligibility rules for registration, not merely peripheral consistency requirements.</t>
+          <t>Registration deadlines and capacity limits are core eligibility rules for registration, not merely peripheral consistency requirements.</t>
         </is>
       </c>
     </row>
@@ -15161,7 +15161,7 @@
       </c>
       <c r="J30" s="8" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what actions must an attendee complete for registration to be considered successful. The stated risk is that the registration scope and completion state are undefined, leaving developers unable to distinguish an initiated registration from a completed one. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what actions must an attendee complete for registration to be considered successful. The stated risk is that the registration scope and completion state are undefined, leaving developers unable to distinguish an initiated registration from a completed one. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K30" s="8" t="inlineStr">
@@ -15181,7 +15181,7 @@
       </c>
       <c r="N30" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The required attendee actions define the primary registration workflow, which is missing from the story.</t>
+          <t>The required attendee actions define the primary registration workflow, which is missing from the story.</t>
         </is>
       </c>
     </row>
@@ -15233,7 +15233,7 @@
       </c>
       <c r="J31" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what user action is intended by “something about see the schedule”. The stated risk is that the wording does not establish the required behavior, preventing a testable definition of successful use. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what user action is intended by “something about see the schedule”. The stated risk is that the wording does not establish the required behavior, preventing a testable definition of successful use. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K31" s="8" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="N31" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): “Something about see the schedule” is linguistically ambiguous about the intended action.</t>
+          <t>“Something about see the schedule” is linguistically ambiguous about the intended action.</t>
         </is>
       </c>
     </row>
@@ -15305,7 +15305,7 @@
       </c>
       <c r="J32" s="8" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what video input must be supported: prerecorded video, a live stream, or both. The stated risk is that the input lifecycle determines whether processing operates on a complete timeline or must handle incoming frames continuously. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what video input must be supported: prerecorded video, a live stream, or both. The stated risk is that the input lifecycle determines whether processing operates on a complete timeline or must handle incoming frames continuously. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K32" s="8" t="inlineStr">
@@ -15325,7 +15325,7 @@
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The input can be prerecorded, live, or both, yielding distinct plausible functional interpretations.</t>
+          <t>The input can be prerecorded, live, or both, yielding distinct plausible functional interpretations.</t>
         </is>
       </c>
     </row>
@@ -15377,7 +15377,7 @@
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules must edited timestamps satisfy regarding video duration, segment order, overlaps, and gaps. The stated risk is that missing validation rules could allow invalid boundaries or reject legitimate corrections. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules must edited timestamps satisfy regarding video duration, segment order, overlaps, and gaps. The stated risk is that missing validation rules could allow invalid boundaries or reject legitimate corrections. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr">
@@ -15397,7 +15397,7 @@
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Overlap, ordering, duration, and gap constraints are precise timestamp validation rules; the question primarily seeks technical boundary conditions.</t>
+          <t>Overlap, ordering, duration, and gap constraints are precise timestamp validation rules; the question primarily seeks technical boundary conditions.</t>
         </is>
       </c>
     </row>
@@ -15449,7 +15449,7 @@
       </c>
       <c r="J34" s="8" t="inlineStr">
         <is>
-          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what results must the counter return, and in what format. The stated risk is that the story does not define the output contract, preventing validation that the results meet the user's intended use. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what results must the counter return, and in what format. The stated risk is that the story does not define the output contract, preventing validation that the results meet the user's intended use. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr">
@@ -15469,7 +15469,7 @@
       </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): The output and its observable format are needed to formulate an acceptance test for the counter.</t>
+          <t>The output and its observable format are needed to formulate an acceptance test for the counter.</t>
         </is>
       </c>
     </row>
@@ -15521,7 +15521,7 @@
       </c>
       <c r="J35" s="8" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which Snapshot Serengeti images must be processed. The stated risk is that the image population is unspecified, leaving processing scope and workload undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which Snapshot Serengeti images must be processed. The stated risk is that the image population is unspecified, leaving processing scope and workload undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
       <c r="K35" s="8" t="inlineStr">
@@ -15541,7 +15541,7 @@
       </c>
       <c r="N35" s="19" t="inlineStr">
         <is>
-          <t>Proposed adjudication (pending joint specialist approval): Both specialists identify the same substantive domain-scope gap; the second anchor contains an apparent spreadsheet artifact, not a different criterion.</t>
+          <t>Both specialists identify the same substantive domain-scope gap; the second anchor contains an apparent spreadsheet artifact, not a different criterion.</t>
         </is>
       </c>
     </row>
@@ -16627,7 +16627,7 @@
       </c>
       <c r="I2" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the user has no profile history. The stated risk is that the required recommendation input may be absent, leaving the initial user experience and expected fallback behavior undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the user has no profile history. The stated risk is that the required recommendation input may be absent, leaving the initial user experience and expected fallback behavior undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -16674,7 +16674,7 @@
       </c>
       <c r="I3" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine whether users are “similar”. The stated risk is that no similarity rule is specified, so developers cannot determine which users qualify or validate their selection. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine whether users are “similar”. The stated risk is that no similarity rule is specified, so developers cannot determine which users qualify or validate their selection. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -16721,7 +16721,7 @@
       </c>
       <c r="I4" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what permission rules govern using other users’ listening paths for music discovery. The stated risk is that the story requires using other users’ listening activity without defining authorized use, leaving data eligibility and privacy boundaries unresolved. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what permission rules govern using other users’ listening paths for music discovery. The stated risk is that the story requires using other users’ listening activity without defining authorized use, leaving data eligibility and privacy boundaries unresolved. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -16909,7 +16909,7 @@
       </c>
       <c r="I8" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criterion determines which eligible news events are “most relevant”. The stated risk is that no ranking criterion is specified, so recommendation ordering and quality cannot be objectively validated. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criterion determines which eligible news events are “most relevant”. The stated risk is that no ranking criterion is specified, so recommendation ordering and quality cannot be objectively validated. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17003,7 +17003,7 @@
       </c>
       <c r="I10" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what geographical relationship determines which videos appear on the map for the user’s location. The stated risk is that the story does not define how videos relate to locations or the geographical scope of matching, leaving content selection and acceptance tests undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what geographical relationship determines which videos appear on the map for the user’s location. The stated risk is that the story does not define how videos relate to locations or the geographical scope of matching, leaving content selection and acceptance tests undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17050,7 +17050,7 @@
       </c>
       <c r="I11" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should the system determine the user’s location when it is unavailable or access to it is denied. The stated risk is that the location dependency lacks a defined fallback, leaving the map’s behavior uncertain when location cannot be obtained. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should the system determine the user’s location when it is unavailable or access to it is denied. The stated risk is that the location dependency lacks a defined fallback, leaving the map’s behavior uncertain when location cannot be obtained. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17144,7 +17144,7 @@
       </c>
       <c r="I13" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the user's location cannot be obtained. The stated risk is that no failure behavior is defined, leaving content access and the map's state unspecified when location is unavailable. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the user's location cannot be obtained. The stated risk is that no failure behavior is defined, leaving content access and the map's state unspecified when location is unavailable. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17238,7 +17238,7 @@
       </c>
       <c r="I15" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which audio and visual quality metrics must admins be able to filter by. The stated risk is that the story names no metrics, leaving the required video attributes and filter criteria undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which audio and visual quality metrics must admins be able to filter by. The stated risk is that the story names no metrics, leaving the required video attributes and filter criteria undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17285,7 +17285,7 @@
       </c>
       <c r="I16" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should filtering treat videos whose selected quality metrics are missing or invalid. The stated risk is that undefined handling of unavailable or unusable metric values could incorrectly include or exclude videos. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should filtering treat videos whose selected quality metrics are missing or invalid. The stated risk is that undefined handling of unavailable or unusable metric values could incorrectly include or exclude videos. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17332,7 +17332,7 @@
       </c>
       <c r="I17" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks must the assessment run before upload, or assess prior editing after the audio has been uploaded. The stated risk is that the wording leaves the processing sequence ambiguous, affecting when audio is available and where assessment belongs in the upload flow. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks must the assessment run before upload, or assess prior editing after the audio has been uploaded. The stated risk is that the wording leaves the processing sequence ambiguous, affecting when audio is available and where assessment belongs in the upload flow. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17379,7 +17379,7 @@
       </c>
       <c r="I18" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which previously approved project policy must the assessment apply, and what rules does it contain. The stated risk is that the policy is absent, so compliance criteria and acceptance tests cannot be defined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which previously approved project policy must the assessment apply, and what rules does it contain. The stated risk is that the policy is absent, so compliance criteria and acceptance tests cannot be defined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17426,7 +17426,7 @@
       </c>
       <c r="I19" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what result must the admin receive when editing history or policy compliance cannot be determined. The stated risk is that undefined handling of inconclusive assessments could present uncertainty as a definitive finding. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what result must the admin receive when editing history or policy compliance cannot be determined. The stated risk is that undefined handling of inconclusive assessments could present uncertainty as a definitive finding. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17473,7 +17473,7 @@
       </c>
       <c r="I20" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which engagement metrics should be calculated, and how is each defined. The stated risk is that neither the metrics nor their calculation rules are specified, preventing consistent implementation and verification. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which engagement metrics should be calculated, and how is each defined. The stated risk is that neither the metrics nor their calculation rules are specified, preventing consistent implementation and verification. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17520,7 +17520,7 @@
       </c>
       <c r="I21" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what constitutes a citizen annotation for measuring engagement. The stated risk is that the annotation unit and qualifying annotation types are undefined, so implementations could count different activities. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what constitutes a citizen annotation for measuring engagement. The stated risk is that the annotation unit and qualifying annotation types are undefined, so implementations could count different activities. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17567,7 +17567,7 @@
       </c>
       <c r="I22" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how should a volunteer’s experience level be determined. The stated risk is that the story does not define the evidence or criteria for experience, so implementations could assign different levels to the same volunteer. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how should a volunteer’s experience level be determined. The stated risk is that the story does not define the evidence or criteria for experience, so implementations could assign different levels to the same volunteer. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17708,7 +17708,7 @@
       </c>
       <c r="I25" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the experience information required for the calculation is unavailable. The stated risk is that missing input behavior is unspecified, leaving developers unable to determine whether a reliability weight can be produced. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when the experience information required for the calculation is unavailable. The stated risk is that missing input behavior is unspecified, leaving developers unable to determine whether a reliability weight can be produced. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17755,7 +17755,7 @@
       </c>
       <c r="I26" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine whether text, an image, or a video is the appropriate way to interrupt. The stated risk is that no decision rules or success criteria are provided, so the choice cannot be implemented or validated. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what criteria determine whether text, an image, or a video is the appropriate way to interrupt. The stated risk is that no decision rules or success criteria are provided, so the choice cannot be implemented or validated. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17802,7 +17802,7 @@
       </c>
       <c r="I27" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks should the feature only report the appropriate format, or also initiate the interruption. The stated risk is that the action boundary is unclear, affecting user flow and whether communication delivery is required. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks should the feature only report the appropriate format, or also initiate the interruption. The stated risk is that the action boundary is unclear, affecting user flow and whether communication delivery is required. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17896,7 +17896,7 @@
       </c>
       <c r="I29" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information should the feature use to make that determination. The stated risk is that required inputs and their sources are unspecified, leaving data requirements and the feasibility of the decision logic unresolved. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information should the feature use to make that determination. The stated risk is that required inputs and their sources are unspecified, leaving data requirements and the feasibility of the decision logic unresolved. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -17990,7 +17990,7 @@
       </c>
       <c r="I31" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what conditions make a subject eligible for a Zoonibot comment. The stated risk is that no commenting criteria are specified, preventing implementation and validation of when a comment is warranted. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what conditions make a subject eligible for a Zoonibot comment. The stated risk is that no commenting criteria are specified, preventing implementation and validation of when a comment is warranted. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18084,7 +18084,7 @@
       </c>
       <c r="I33" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which aspects of a volunteer’s previous experiences should determine project recommendations. The stated risk is that the story does not define the experience data required, leaving recommendation inputs and volunteer data requirements uncertain. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which aspects of a volunteer’s previous experiences should determine project recommendations. The stated risk is that the story does not define the experience data required, leaving recommendation inputs and volunteer data requirements uncertain. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18131,7 +18131,7 @@
       </c>
       <c r="I34" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which projects are eligible to be recommended to a volunteer. The stated risk is that the eligible project set is undefined, creating a risk of recommending projects that the volunteer cannot participate in. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which projects are eligible to be recommended to a volunteer. The stated risk is that the eligible project set is undefined, creating a risk of recommending projects that the volunteer cannot participate in. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18272,7 +18272,7 @@
       </c>
       <c r="I37" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what constraints apply to the optional description, and how should an omitted or blank description be treated. The stated risk is that description validation and the meaning of an empty value are undefined, risking inconsistent acceptance and storage. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what constraints apply to the optional description, and how should an omitted or blank description be treated. The stated risk is that description validation and the meaning of an empty value are undefined, risking inconsistent acceptance and storage. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18366,7 +18366,7 @@
       </c>
       <c r="I39" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks is the invitation URL specific to a game, an individual estimator, or both. The stated risk is that the URL’s scope determines how the system identifies the intended game and recipient and prevents unintended access. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks is the invitation URL specific to a game, an individual estimator, or both. The stated risk is that the URL’s scope determines how the system identifies the intended game and recipient and prevents unintended access. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18413,7 +18413,7 @@
       </c>
       <c r="I40" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks under what conditions does an invitation URL become invalid. The stated risk is that invitation validity is undefined, preventing consistent handling and testing of expired or otherwise unusable links. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks under what conditions does an invitation URL become invalid. The stated risk is that invitation validity is undefined, preventing consistent handling and testing of expired or otherwise unusable links. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18554,7 +18554,7 @@
       </c>
       <c r="I43" s="16" t="inlineStr">
         <is>
-          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what action should the moderator be able to perform. The stated risk is that the story omits the requested capability, so the moderator’s workflow and functional behavior cannot be determined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The clarification concerns an undefined user-visible action, result, or functional boundary. Specifically, the question asks what action should the moderator be able to perform. The stated risk is that the story omits the requested capability, so the moderator’s workflow and functional behavior cannot be determined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18742,7 +18742,7 @@
       </c>
       <c r="I47" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which moderators are authorized to edit a particular item. The stated risk is that the authorization scope is unspecified, risking unauthorized changes to items outside a moderator’s responsibility. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which moderators are authorized to edit a particular item. The stated risk is that the authorization scope is unspecified, risking unauthorized changes to items outside a moderator’s responsibility. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18883,7 +18883,7 @@
       </c>
       <c r="I50" s="16" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks if an item already has estimation data, what should happen to that data when the item is deleted. The stated risk is that the treatment of potentially associated data is undefined, risking orphaned records or unintended loss of estimates. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks if an item already has estimation data, what should happen to that data when the item is deleted. The stated risk is that the treatment of potentially associated data is undefined, risking orphaned records or unintended loss of estimates. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -18977,7 +18977,7 @@
       </c>
       <c r="I52" s="16" t="inlineStr">
         <is>
-          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what unit and allowed values must the estimate use. The stated risk is that the estimate’s representation is unspecified, preventing consistent storage and input validation. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question requests precise input constraints or validation parameters. Specifically, the question asks what unit and allowed values must the estimate use. The stated risk is that the estimate’s representation is unspecified, preventing consistent storage and input validation. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19071,7 +19071,7 @@
       </c>
       <c r="I54" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks at what stage of a game must its transcript be available for viewing. The stated risk is that availability during or after a game is undefined, leaving transcript lifecycle and update behavior uncertain. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks at what stage of a game must its transcript be available for viewing. The stated risk is that availability during or after a game is undefined, leaving transcript lifecycle and update behavior uncertain. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19118,7 +19118,7 @@
       </c>
       <c r="I55" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how does the user identify which game’s transcript to view. The stated risk is that the target-game selection flow is unspecified, preventing implementation and validation of the viewing journey. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how does the user identify which game’s transcript to view. The stated risk is that the target-game selection flow is unspecified, preventing implementation and validation of the viewing journey. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19212,7 +19212,7 @@
       </c>
       <c r="I57" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information must a game transcript contain. The stated risk is that undefined transcript contents prevent determining which game data must be exported and testing completeness. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information must a game transcript contain. The stated risk is that undefined transcript contents prevent determining which game data must be exported and testing completeness. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19306,7 +19306,7 @@
       </c>
       <c r="I59" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what is the authoritative source of the sponsor list. The stated risk is that the story does not identify where sponsor records originate, leaving data retrieval and correctness validation undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what is the authoritative source of the sponsor list. The stated risk is that the story does not identify where sponsor records originate, leaving data retrieval and correctness validation undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19353,7 +19353,7 @@
       </c>
       <c r="I60" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should an anonymous user see when the sponsor list is empty or cannot be retrieved. The stated risk is that empty and failure behavior are unspecified, preventing consistent handling and verification of these distinct outcomes. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should an anonymous user see when the sponsor list is empty or cannot be retrieved. The stated risk is that empty and failure behavior are unspecified, preventing consistent handling and verification of these distinct outcomes. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19400,7 +19400,7 @@
       </c>
       <c r="I61" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which user profiles and profile fields may an anonymous user view. The stated risk is that the list’s scope and visible data are unspecified, preventing access-control and privacy requirements from being tested. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which user profiles and profile fields may an anonymous user view. The stated risk is that the list’s scope and visible data are unspecified, preventing access-control and privacy requirements from being tested. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19447,7 +19447,7 @@
       </c>
       <c r="I62" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what must anonymous users see when the profile list cannot be retrieved. The stated risk is that retrieval failure behavior is undefined, so users could receive a misleading empty list or an indefinite loading state. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what must anonymous users see when the profile list cannot be retrieved. The stated risk is that retrieval failure behavior is undefined, so users could receive a misleading empty list or an indefinite loading state. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19494,7 +19494,7 @@
       </c>
       <c r="I63" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what spatial information must the map show to locate buildings and rooms. The stated risk is that the story does not specify whether room locations require floor identification, interior layouts, or other spatial relationships, leaving the map’s data requirements uncertain. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what spatial information must the map show to locate buildings and rooms. The stated risk is that the story does not specify whether room locations require floor identification, interior layouts, or other spatial relationships, leaving the map’s data requirements uncertain. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19541,7 +19541,7 @@
       </c>
       <c r="I64" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks does a waitlist entry apply to an entire training or to a particular scheduled session. The stated risk is that the waitlist’s scope is undefined, risking enrollment against the wrong training occurrence. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks does a waitlist entry apply to an entire training or to a particular scheduled session. The stated risk is that the waitlist’s scope is undefined, risking enrollment against the wrong training occurrence. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19588,7 +19588,7 @@
       </c>
       <c r="I65" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what determines the “appropriate order” of trainings, including how ties are resolved. The stated risk is that no ordering rule is defined, so developers cannot implement or test the intended sequence. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what determines the “appropriate order” of trainings, including how ties are resolved. The stated risk is that no ordering rule is defined, so developers cannot implement or test the intended sequence. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19635,7 +19635,7 @@
       </c>
       <c r="I66" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the trainee see when the prerequisite has not been completed. The stated risk is that the blocked state is unspecified, leaving developers unable to determine the required interface behavior or validate that the visibility restriction is satisfied. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the trainee see when the prerequisite has not been completed. The stated risk is that the blocked state is unspecified, leaving developers unable to determine the required interface behavior or validate that the visibility restriction is satisfied. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19682,7 +19682,7 @@
       </c>
       <c r="I67" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule determines whether two venue records are duplicates. The stated risk is that undefined identity and uniqueness rules could allow duplicate venues or reject distinct venues. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rule determines whether two venue records are duplicates. The stated risk is that undefined identity and uniqueness rules could allow duplicate venues or reject distinct venues. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19729,7 +19729,7 @@
       </c>
       <c r="I68" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information is required to create a venue. The stated risk is that missing required attributes prevent defining the data model and testing whether a venue record is complete. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information is required to create a venue. The stated risk is that missing required attributes prevent defining the data model and testing whether a venue record is complete. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19776,7 +19776,7 @@
       </c>
       <c r="I69" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules does the previously approved project policy impose on creating and maintaining venues. The stated risk is that the referenced policy is absent, so policy compliance cannot be implemented or verified. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what rules does the previously approved project policy impose on creating and maintaining venues. The stated risk is that the referenced policy is absent, so policy compliance cannot be implemented or verified. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19823,7 +19823,7 @@
       </c>
       <c r="I70" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how does an anonymous user identify the venue whose details they want to view. The stated risk is that the entry point and venue selection flow are unspecified, leaving the viewing journey incomplete. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks how does an anonymous user identify the venue whose details they want to view. The stated risk is that the entry point and venue selection flow are unspecified, leaving the viewing journey incomplete. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -19917,7 +19917,7 @@
       </c>
       <c r="I72" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which venues must a training coordinator be able to view. The stated risk is that the eligible venue set is unspecified, preventing definition of retrieval scope and tests for venue inclusion or exclusion. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which venues must a training coordinator be able to view. The stated risk is that the eligible venue set is unspecified, preventing definition of retrieval scope and tests for venue inclusion or exclusion. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20011,7 +20011,7 @@
       </c>
       <c r="I74" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the administrator experience when a blog post cannot be saved. The stated risk is that failure behavior and preservation of entered content are unspecified, risking silent failures, lost work, or duplicate posts during retries. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the administrator experience when a blog post cannot be saved. The stated risk is that failure behavior and preservation of entered content are unspecified, risking silent failures, lost work, or duplicate posts during retries. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20058,7 +20058,7 @@
       </c>
       <c r="I75" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what content is required for a valid blog post. The stated risk is that required fields and content constraints are unspecified, preventing definition of the data model and validation criteria. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what content is required for a valid blog post. The stated risk is that required fields and content constraints are unspecified, preventing definition of the data model and validation criteria. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20105,7 +20105,7 @@
       </c>
       <c r="I76" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks who qualifies as a sponsor, and what determines their permission to create blog posts. The stated risk is that the actor and authorization rules are undefined, so eligibility checks and access-control tests cannot be established. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks who qualifies as a sponsor, and what determines their permission to create blog posts. The stated risk is that the actor and authorization rules are undefined, so eligibility checks and access-control tests cannot be established. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20152,7 +20152,7 @@
       </c>
       <c r="I77" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information must a blog post contain to be created successfully. The stated risk is that required content and attributes are unspecified, preventing a defined data model and testable creation criteria. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what information must a blog post contain to be created successfully. The stated risk is that required content and attributes are unspecified, preventing a defined data model and testable creation criteria. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20293,7 +20293,7 @@
       </c>
       <c r="I80" s="16" t="inlineStr">
         <is>
-          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what outcome marks registration as successfully completed. The stated risk is that the story provides no observable completion criterion, so implementation and tests cannot distinguish a submitted request from a completed registration. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what outcome marks registration as successfully completed. The stated risk is that the story provides no observable completion criterion, so implementation and tests cannot distinguish a submitted request from a completed registration. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20340,7 +20340,7 @@
       </c>
       <c r="I81" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what schedule does “the schedule” refer to. The stated risk is that the schedule’s subject and source are undefined, so developers cannot determine which data to retrieve. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what schedule does “the schedule” refer to. The stated risk is that the schedule’s subject and source are undefined, so developers cannot determine which data to retrieve. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20481,7 +20481,7 @@
       </c>
       <c r="I84" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what should each music recommendation contain. The stated risk is that the recommended entity and required output information are unspecified, leaving the result data model and acceptance criteria undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what should each music recommendation contain. The stated risk is that the recommended entity and required output information are unspecified, leaving the result data model and acceptance criteria undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20528,7 +20528,7 @@
       </c>
       <c r="I85" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which music catalog should supply the recommendations. The stated risk is that the source and boundaries of eligible music are unspecified, leaving data availability and external dependencies unresolved. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which music catalog should supply the recommendations. The stated risk is that the source and boundaries of eligible music are unspecified, leaving data availability and external dependencies unresolved. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20575,7 +20575,7 @@
       </c>
       <c r="I86" s="16" t="inlineStr">
         <is>
-          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what observable condition establishes that the prerequisite story has been completed. The stated risk is that “Completed” lacks a testable definition, leaving the upload eligibility rule undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what observable condition establishes that the prerequisite story has been completed. The stated risk is that “Completed” lacks a testable definition, leaving the upload eligibility rule undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20622,7 +20622,7 @@
       </c>
       <c r="I87" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when a user attempts to upload an image before the prerequisite is completed. The stated risk is that the blocked interaction and failure response are unspecified, preventing consistent enforcement and acceptance testing. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should happen when a user attempts to upload an image before the prerequisite is completed. The stated risk is that the blocked interaction and failure response are unspecified, preventing consistent enforcement and acceptance testing. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20669,7 +20669,7 @@
       </c>
       <c r="I88" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which users’ credentials may an admin manage. The stated risk is that the authorization scope is unspecified, risking unauthorized changes to credentials. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which users’ credentials may an admin manage. The stated risk is that the authorization scope is unspecified, risking unauthorized changes to credentials. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20716,7 +20716,7 @@
       </c>
       <c r="I89" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what defines a segmentation boundary in a video. The stated risk is that without a definition, developers cannot determine which detected points qualify as boundaries or validate segmentation correctness. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what defines a segmentation boundary in a video. The stated risk is that without a definition, developers cannot determine which detected points qualify as boundaries or validate segmentation correctness. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20763,7 +20763,7 @@
       </c>
       <c r="I90" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks must this feature generate automated segmentation boundaries, or display boundaries already produced elsewhere. The stated risk is that the story does not establish whether automated segmentation processing is part of the feature, leaving its scope and dependencies undefined. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks must this feature generate automated segmentation boundaries, or display boundaries already produced elsewhere. The stated risk is that the story does not establish whether automated segmentation processing is part of the feature, leaving its scope and dependencies undefined. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20810,7 +20810,7 @@
       </c>
       <c r="I91" s="16" t="inlineStr">
         <is>
-          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what maximum elapsed time is acceptable from the admin requesting the boundaries to their being visible. The stated risk is that “As fast as necessary” supplies no measurable performance target, making response-time acceptance tests impossible to define. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The expected observable result is insufficiently specified to derive a reliable acceptance test. Specifically, the question asks what maximum elapsed time is acceptable from the admin requesting the boundaries to their being visible. The stated risk is that “As fast as necessary” supplies no measurable performance target, making response-time acceptance tests impossible to define. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20857,7 +20857,7 @@
       </c>
       <c r="I92" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the admin see when automated segmentation boundaries are unavailable. The stated risk is that the missing unavailable-result behavior could cause an unprocessed video or failed segmentation to appear indistinguishable from a valid result with no boundaries. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what should the admin see when automated segmentation boundaries are unavailable. The stated risk is that the missing unavailable-result behavior could cause an unprocessed video or failed segmentation to appear indistinguishable from a valid result with no boundaries. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20904,7 +20904,7 @@
       </c>
       <c r="I93" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what constitutes a segmentation boundary in this story. The stated risk is that the boundary’s meaning is undefined, leaving its data representation and acceptance criteria uncertain. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks what constitutes a segmentation boundary in this story. The stated risk is that the boundary’s meaning is undefined, leaving its data representation and acceptance criteria uncertain. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -20951,7 +20951,7 @@
       </c>
       <c r="I94" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what must happen when a clip fails validation. The stated risk is that the failure outcome and subsequent workflow are unspecified, leaving unsuccessful validation without defined behavior. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks what must happen when a clip fails validation. The stated risk is that the failure outcome and subsequent workflow are unspecified, leaving unsuccessful validation without defined behavior. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -21045,7 +21045,7 @@
       </c>
       <c r="I96" s="16" t="inlineStr">
         <is>
-          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which timestamps should the user be able to edit for each segment. The stated risk is that the editable timestamp fields are unspecified, preventing definition of the editing controls and update behavior. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>A domain-specific rule or definition necessary to implement the requested behavior is missing. Specifically, the question asks which timestamps should the user be able to edit for each segment. The stated risk is that the editable timestamp fields are unspecified, preventing definition of the editing controls and update behavior. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -21092,7 +21092,7 @@
       </c>
       <c r="I97" s="16" t="inlineStr">
         <is>
-          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks when further contrasting annotations arrive for an already alerted subject, should another alert be generated. The stated risk is that undefined repeat-trigger behavior could produce duplicate alerts or suppress subsequent conflicts. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns downstream consistency, lifecycle restrictions, or preservation of related records. Specifically, the question asks when further contrasting annotations arrive for an already alerted subject, should another alert be generated. The stated risk is that undefined repeat-trigger behavior could produce duplicate alerts or suppress subsequent conflicts. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -21139,7 +21139,7 @@
       </c>
       <c r="I98" s="16" t="inlineStr">
         <is>
-          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what should happen to an image when it is automatically “isolated”. The stated risk is that “Isolate” does not define the required action or the image’s resulting availability, leaving the core behavior untestable. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The story admits competing interpretations of the requested behavior. Specifically, the question asks what should happen to an image when it is automatically “isolated”. The stated risk is that “Isolate” does not define the required action or the image’s resulting availability, leaving the core behavior untestable. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -21186,7 +21186,7 @@
       </c>
       <c r="I99" s="16" t="inlineStr">
         <is>
-          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should the system handle images whose animal presence cannot be determined confidently. The stated risk is that undefined handling of uncertain images could isolate images containing animals or leave qualifying images unprocessed. This supports the selected protocol anchor; the classification is a provisional judgment for specialist review.</t>
+          <t>The question concerns a missing-data, invalid-state, or failure-handling path. Specifically, the question asks how should the system handle images whose animal presence cannot be determined confidently. The stated risk is that undefined handling of uncertain images could isolate images containing animals or leave qualifying images unprocessed. This supports the selected protocol anchor.</t>
         </is>
       </c>
     </row>
@@ -22269,7 +22269,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>All original worksheets and values are preserved as received, including provisional notes and proposed consensus wording. These describe the historical draft, not an outstanding review status.</t>
+          <t>Earlier coding worksheets are historical; Final contains the consensus labels.</t>
         </is>
       </c>
     </row>
@@ -22317,7 +22317,7 @@
       </c>
       <c r="B10" s="22" t="inlineStr">
         <is>
-          <t>Documentation updated from researcher confirmation; no new classification was performed in this update.</t>
+          <t>The review record documents the human consensus classification.</t>
         </is>
       </c>
     </row>

</xml_diff>